<commit_message>
[PO] - import data using purchase price
</commit_message>
<xml_diff>
--- a/public/upload/template/po_pembelian_template.xlsx
+++ b/public/upload/template/po_pembelian_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\jez_pro\public\upload\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IT1\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C22C2A51-2D84-4960-83A3-220D628975FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5789D5E-97EB-44E9-B031-8547BA709511}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{55DBDE80-1256-4436-8BF1-96AF70A082A5}"/>
+    <workbookView xWindow="22932" yWindow="-84" windowWidth="23256" windowHeight="12456" xr2:uid="{4D4CC1C9-A36D-4256-88BC-9010A5D112FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,10 +23,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,10 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>SPSARD12041</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>SKU</t>
   </si>
@@ -45,66 +39,56 @@
     <t>DISC</t>
   </si>
   <si>
+    <t>EX DISC</t>
+  </si>
+  <si>
     <t>SUB DISC</t>
   </si>
   <si>
     <t>QTY</t>
   </si>
   <si>
-    <t>* isi Discount sesuai dengan kebutuhan , jika tidak ada discount tetap di tulis dengan angka 0</t>
-  </si>
-  <si>
-    <t>EX DISC</t>
+    <t>JK26PORA20</t>
+  </si>
+  <si>
+    <t>JK26ITAH26</t>
+  </si>
+  <si>
+    <t>JK25BMU326</t>
+  </si>
+  <si>
+    <t>SDPAT1036</t>
+  </si>
+  <si>
+    <t>SDPAT1136</t>
+  </si>
+  <si>
+    <t>SDPAT1137</t>
+  </si>
+  <si>
+    <t>Hbeli</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -119,13 +103,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,53 +418,152 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{140FE099-81DA-4018-87F3-CA35D8FB4585}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C6A881-2338-45F1-BFBA-9D97D61CAC99}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>12</v>
+      </c>
+      <c r="F2">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>24</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>36</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
         <v>30</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="H4" s="3"/>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>30</v>
+      </c>
+      <c r="E5">
+        <v>48</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>72</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>